<commit_message>
Add drop-down lists to the curriculum workbook
Status, Claude confidence and Audio columns on the Words and Sentences
tabs now offer their allowed values, so a typo can't throw off the
Progress counts; the header rows are frozen, and the Read me says how to
name and upload recordings.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curriculum/a1-english-speakers.xlsx
+++ b/curriculum/a1-english-speakers.xlsx
@@ -609,7 +609,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>7. Audio: put Y when a native speaker has recorded the word or sentence.</t>
+          <t>7. Audio: record on your own device, name the file after the row ID (W001.m4a, S001.m4a), upload it in the admin, then set Audio to Y.</t>
         </is>
       </c>
     </row>
@@ -21702,11 +21702,23 @@
       <c r="Q269" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="M2:N269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="6">
+    <dataValidation sqref="K2:K269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,Draft,Reviewed,Needs change"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:P269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To do,Draft,Reviewed,Needs change"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P269" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -26404,11 +26416,23 @@
       <c r="T67" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="P2:Q67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="6">
+    <dataValidation sqref="N2:N67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,Draft,Reviewed,Needs change"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:S67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"To do,Draft,Reviewed,Needs change"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>